<commit_message>
feat: add Excel report generation services and templates for RTL, RTM, and quality standards
</commit_message>
<xml_diff>
--- a/resources/templates/Laporan Pelaksanaan Perkuliahan Prodi Ilmu Komputer.xlsx
+++ b/resources/templates/Laporan Pelaksanaan Perkuliahan Prodi Ilmu Komputer.xlsx
@@ -1272,1001 +1272,642 @@
       <c r="H16" s="5"/>
       <c r="I16" s="20"/>
     </row>
-    <row r="17" spans="1:9" s="4" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="20"/>
-    </row>
-    <row r="18" spans="1:9" s="4" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="5"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="20"/>
-    </row>
-    <row r="19" spans="1:9" s="4" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="5"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="20"/>
-    </row>
-    <row r="20" spans="1:9" s="4" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="45"/>
-      <c r="B20" s="46"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="48"/>
-    </row>
-    <row r="21" spans="1:9" s="4" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="45"/>
-      <c r="B21" s="46"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="47"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="48"/>
-    </row>
-    <row r="22" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="45"/>
-      <c r="B22" s="46"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
-    </row>
-    <row r="23" spans="1:9" s="4" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="45"/>
-      <c r="B23" s="46"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="48"/>
-    </row>
-    <row r="24" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="45"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="45"/>
-    </row>
-    <row r="25" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="45"/>
-      <c r="B25" s="46"/>
-      <c r="C25" s="45"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="45"/>
-      <c r="I25" s="45"/>
-    </row>
-    <row r="26" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="45"/>
-      <c r="B26" s="46"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="45"/>
-      <c r="I26" s="45"/>
-    </row>
-    <row r="27" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="45"/>
-      <c r="B27" s="46"/>
-      <c r="C27" s="45"/>
-      <c r="D27" s="46"/>
-      <c r="E27" s="45"/>
-      <c r="F27" s="45"/>
-      <c r="G27" s="45"/>
-      <c r="H27" s="45"/>
-      <c r="I27" s="45"/>
-    </row>
-    <row r="28" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="45"/>
-      <c r="B28" s="46"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="45"/>
-      <c r="G28" s="45"/>
-      <c r="H28" s="45"/>
-      <c r="I28" s="45"/>
-    </row>
-    <row r="29" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="45"/>
-      <c r="B29" s="46"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="45"/>
-    </row>
-    <row r="30" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="45"/>
-      <c r="B30" s="46"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="51"/>
-      <c r="G30" s="45"/>
-      <c r="H30" s="45"/>
-      <c r="I30" s="45"/>
-    </row>
-    <row r="31" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="45"/>
-      <c r="B31" s="46"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="46"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="51"/>
-      <c r="G31" s="45"/>
-      <c r="H31" s="45"/>
-      <c r="I31" s="45"/>
-    </row>
-    <row r="32" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="45"/>
-      <c r="B32" s="46"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="51"/>
-      <c r="G32" s="45"/>
-      <c r="H32" s="45"/>
-      <c r="I32" s="45"/>
-    </row>
-    <row r="33" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="45"/>
-      <c r="B33" s="46"/>
-      <c r="C33" s="45"/>
-      <c r="D33" s="46"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="45"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="45"/>
-    </row>
-    <row r="34" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="45"/>
-      <c r="B34" s="46"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="45"/>
-      <c r="H34" s="45"/>
-      <c r="I34" s="45"/>
-    </row>
-    <row r="35" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="45"/>
-      <c r="B35" s="46"/>
-      <c r="C35" s="45"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-    </row>
-    <row r="36" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="45"/>
-      <c r="B36" s="46"/>
-      <c r="C36" s="45"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="45"/>
-      <c r="F36" s="45"/>
-      <c r="G36" s="45"/>
-      <c r="H36" s="45"/>
-      <c r="I36" s="45"/>
-    </row>
-    <row r="37" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="45"/>
-      <c r="B37" s="46"/>
-      <c r="C37" s="45"/>
-      <c r="D37" s="46"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="45"/>
-      <c r="H37" s="45"/>
-      <c r="I37" s="45"/>
-    </row>
-    <row r="38" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="45"/>
-      <c r="B38" s="46"/>
-      <c r="C38" s="45"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="45"/>
-      <c r="G38" s="45"/>
-      <c r="H38" s="45"/>
-      <c r="I38" s="45"/>
-    </row>
-    <row r="39" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="45"/>
-      <c r="B39" s="46"/>
-      <c r="C39" s="45"/>
-      <c r="D39" s="46"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
-      <c r="H39" s="45"/>
-      <c r="I39" s="45"/>
-    </row>
-    <row r="40" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="45"/>
-      <c r="B40" s="46"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="46"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="45"/>
-    </row>
-    <row r="41" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="45"/>
-      <c r="B41" s="46"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="46"/>
-      <c r="E41" s="45"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="45"/>
-      <c r="I41" s="45"/>
-    </row>
-    <row r="42" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="45"/>
-      <c r="B42" s="46"/>
-      <c r="C42" s="45"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="45"/>
-      <c r="G42" s="45"/>
-      <c r="H42" s="45"/>
-      <c r="I42" s="45"/>
-    </row>
-    <row r="43" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="45"/>
-      <c r="B43" s="46"/>
-      <c r="C43" s="45"/>
-      <c r="D43" s="46"/>
-      <c r="E43" s="45"/>
-      <c r="F43" s="45"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="45"/>
-      <c r="I43" s="45"/>
-    </row>
-    <row r="44" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="45"/>
-      <c r="B44" s="46"/>
-      <c r="C44" s="45"/>
-      <c r="D44" s="46"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="45"/>
-      <c r="G44" s="45"/>
-      <c r="H44" s="45"/>
-      <c r="I44" s="45"/>
-    </row>
-    <row r="45" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="45"/>
-      <c r="B45" s="46"/>
-      <c r="C45" s="45"/>
-      <c r="D45" s="46"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
-      <c r="G45" s="45"/>
-      <c r="H45" s="45"/>
-      <c r="I45" s="45"/>
-    </row>
-    <row r="46" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="45"/>
-      <c r="B46" s="46"/>
-      <c r="C46" s="45"/>
-      <c r="D46" s="46"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="45"/>
-      <c r="G46" s="45"/>
-      <c r="H46" s="45"/>
-      <c r="I46" s="45"/>
-    </row>
-    <row r="47" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="45"/>
-      <c r="B47" s="46"/>
-      <c r="C47" s="45"/>
-      <c r="D47" s="46"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="45"/>
-      <c r="G47" s="45"/>
-      <c r="H47" s="45"/>
-      <c r="I47" s="45"/>
-    </row>
-    <row r="48" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="45"/>
-      <c r="B48" s="46"/>
-      <c r="C48" s="45"/>
-      <c r="D48" s="46"/>
-      <c r="E48" s="45"/>
-      <c r="F48" s="45"/>
-      <c r="G48" s="45"/>
-      <c r="H48" s="45"/>
-      <c r="I48" s="45"/>
-    </row>
-    <row r="49" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="45"/>
-      <c r="B49" s="46"/>
-      <c r="C49" s="45"/>
-      <c r="D49" s="46"/>
-      <c r="E49" s="45"/>
-      <c r="F49" s="51"/>
-      <c r="G49" s="45"/>
-      <c r="H49" s="45"/>
-      <c r="I49" s="45"/>
-    </row>
-    <row r="50" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="45"/>
-      <c r="B50" s="46"/>
-      <c r="C50" s="45"/>
-      <c r="D50" s="46"/>
-      <c r="E50" s="45"/>
-      <c r="F50" s="51"/>
-      <c r="G50" s="45"/>
-      <c r="H50" s="45"/>
-      <c r="I50" s="45"/>
-    </row>
-    <row r="51" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="45"/>
-      <c r="B51" s="46"/>
-      <c r="C51" s="45"/>
-      <c r="D51" s="46"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="51"/>
-      <c r="G51" s="45"/>
-      <c r="H51" s="45"/>
-      <c r="I51" s="45"/>
-    </row>
-    <row r="52" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="45"/>
-      <c r="B52" s="46"/>
-      <c r="C52" s="45"/>
-      <c r="D52" s="46"/>
-      <c r="E52" s="45"/>
-      <c r="F52" s="45"/>
-      <c r="G52" s="45"/>
-      <c r="H52" s="45"/>
-      <c r="I52" s="45"/>
-    </row>
-    <row r="53" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="45"/>
-      <c r="B53" s="46"/>
-      <c r="C53" s="45"/>
-      <c r="D53" s="46"/>
-      <c r="E53" s="45"/>
-      <c r="F53" s="45"/>
-      <c r="G53" s="45"/>
-      <c r="H53" s="45"/>
-      <c r="I53" s="45"/>
-    </row>
-    <row r="54" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="45"/>
-      <c r="B54" s="46"/>
-      <c r="C54" s="45"/>
-      <c r="D54" s="46"/>
-      <c r="E54" s="45"/>
-      <c r="F54" s="45"/>
-      <c r="G54" s="45"/>
-      <c r="H54" s="45"/>
-      <c r="I54" s="45"/>
-    </row>
-    <row r="55" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="45"/>
-      <c r="B55" s="46"/>
-      <c r="C55" s="45"/>
-      <c r="D55" s="46"/>
-      <c r="E55" s="45"/>
-      <c r="F55" s="45"/>
-      <c r="G55" s="45"/>
-      <c r="H55" s="45"/>
-      <c r="I55" s="45"/>
-    </row>
-    <row r="56" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="45"/>
-      <c r="B56" s="46"/>
-      <c r="C56" s="45"/>
-      <c r="D56" s="46"/>
-      <c r="E56" s="45"/>
-      <c r="F56" s="45"/>
-      <c r="G56" s="45"/>
-      <c r="H56" s="45"/>
-      <c r="I56" s="45"/>
-    </row>
-    <row r="57" spans="1:9" s="4" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="45"/>
-      <c r="B57" s="46"/>
-      <c r="C57" s="45"/>
-      <c r="D57" s="46"/>
-      <c r="E57" s="45"/>
-      <c r="F57" s="45"/>
-      <c r="G57" s="45"/>
-      <c r="H57" s="45"/>
-      <c r="I57" s="45"/>
-    </row>
-    <row r="58" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="45"/>
-      <c r="B58" s="46"/>
-      <c r="C58" s="45"/>
-      <c r="D58" s="46"/>
-      <c r="E58" s="45"/>
-      <c r="F58" s="51"/>
-      <c r="G58" s="45"/>
-      <c r="H58" s="45"/>
-      <c r="I58" s="45"/>
-    </row>
-    <row r="59" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="45"/>
-      <c r="B59" s="46"/>
-      <c r="C59" s="45"/>
-      <c r="D59" s="46"/>
-      <c r="E59" s="45"/>
-      <c r="F59" s="51"/>
-      <c r="G59" s="45"/>
-      <c r="H59" s="45"/>
-      <c r="I59" s="45"/>
-    </row>
-    <row r="60" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="45"/>
-      <c r="B60" s="46"/>
-      <c r="C60" s="45"/>
-      <c r="D60" s="46"/>
-      <c r="E60" s="45"/>
-      <c r="F60" s="51"/>
-      <c r="G60" s="45"/>
-      <c r="H60" s="45"/>
-      <c r="I60" s="45"/>
-    </row>
-    <row r="61" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="45"/>
-      <c r="B61" s="46"/>
-      <c r="C61" s="45"/>
-      <c r="D61" s="46"/>
-      <c r="E61" s="45"/>
-      <c r="F61" s="45"/>
-      <c r="G61" s="45"/>
-      <c r="H61" s="45"/>
-      <c r="I61" s="45"/>
-    </row>
-    <row r="62" spans="1:9" s="4" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="45"/>
-      <c r="B62" s="46"/>
-      <c r="C62" s="45"/>
-      <c r="D62" s="46"/>
-      <c r="E62" s="45"/>
-      <c r="F62" s="51"/>
-      <c r="G62" s="45"/>
-      <c r="H62" s="45"/>
-      <c r="I62" s="48"/>
-    </row>
-    <row r="63" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="45"/>
-      <c r="B63" s="46"/>
-      <c r="C63" s="45"/>
-      <c r="D63" s="46"/>
-      <c r="E63" s="45"/>
-      <c r="F63" s="45"/>
-      <c r="G63" s="45"/>
-      <c r="H63" s="45"/>
-      <c r="I63" s="45"/>
-    </row>
-    <row r="64" spans="1:9" s="4" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="45"/>
-      <c r="B64" s="46"/>
-      <c r="C64" s="45"/>
-      <c r="D64" s="46"/>
-      <c r="E64" s="45"/>
-      <c r="F64" s="45"/>
-      <c r="G64" s="45"/>
-      <c r="H64" s="45"/>
-      <c r="I64" s="45"/>
-    </row>
-    <row r="65" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="45"/>
-      <c r="B65" s="46"/>
-      <c r="C65" s="45"/>
-      <c r="D65" s="46"/>
-      <c r="E65" s="45"/>
-      <c r="F65" s="45"/>
-      <c r="G65" s="45"/>
-      <c r="H65" s="45"/>
-      <c r="I65" s="45"/>
-    </row>
-    <row r="66" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="45"/>
-      <c r="B66" s="46"/>
-      <c r="C66" s="45"/>
-      <c r="D66" s="46"/>
-      <c r="E66" s="45"/>
-      <c r="F66" s="45"/>
-      <c r="G66" s="45"/>
-      <c r="H66" s="45"/>
-      <c r="I66" s="45"/>
-    </row>
-    <row r="67" spans="1:9" s="4" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="45"/>
-      <c r="B67" s="46"/>
-      <c r="C67" s="45"/>
-      <c r="D67" s="46"/>
-      <c r="E67" s="45"/>
-      <c r="F67" s="51"/>
-      <c r="G67" s="45"/>
-      <c r="H67" s="45"/>
-      <c r="I67" s="48"/>
-    </row>
-    <row r="68" spans="1:9" s="4" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="45"/>
-      <c r="B68" s="46"/>
-      <c r="C68" s="45"/>
-      <c r="D68" s="46"/>
-      <c r="E68" s="45"/>
-      <c r="F68" s="51"/>
-      <c r="G68" s="45"/>
-      <c r="H68" s="45"/>
-      <c r="I68" s="48"/>
-    </row>
-    <row r="69" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="45"/>
-      <c r="B69" s="46"/>
-      <c r="C69" s="45"/>
-      <c r="D69" s="46"/>
-      <c r="E69" s="45"/>
-      <c r="F69" s="45"/>
-      <c r="G69" s="45"/>
-      <c r="H69" s="45"/>
-      <c r="I69" s="45"/>
-    </row>
-    <row r="70" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="45"/>
-      <c r="B70" s="46"/>
-      <c r="C70" s="45"/>
-      <c r="D70" s="46"/>
-      <c r="E70" s="45"/>
-      <c r="F70" s="45"/>
-      <c r="G70" s="45"/>
-      <c r="H70" s="45"/>
-      <c r="I70" s="45"/>
-    </row>
-    <row r="71" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="45"/>
-      <c r="B71" s="46"/>
-      <c r="C71" s="45"/>
-      <c r="D71" s="46"/>
-      <c r="E71" s="45"/>
-      <c r="F71" s="51"/>
-      <c r="G71" s="45"/>
-      <c r="H71" s="45"/>
-      <c r="I71" s="45"/>
-    </row>
-    <row r="72" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="45"/>
-      <c r="B72" s="46"/>
-      <c r="C72" s="45"/>
-      <c r="D72" s="46"/>
-      <c r="E72" s="45"/>
-      <c r="F72" s="51"/>
-      <c r="G72" s="45"/>
-      <c r="H72" s="45"/>
-      <c r="I72" s="45"/>
-    </row>
-    <row r="73" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="45"/>
-      <c r="B73" s="46"/>
-      <c r="C73" s="45"/>
-      <c r="D73" s="46"/>
-      <c r="E73" s="45"/>
-      <c r="F73" s="45"/>
-      <c r="G73" s="45"/>
-      <c r="H73" s="45"/>
-      <c r="I73" s="45"/>
-    </row>
-    <row r="74" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="45"/>
-      <c r="B74" s="46"/>
-      <c r="C74" s="45"/>
-      <c r="D74" s="46"/>
-      <c r="E74" s="45"/>
-      <c r="F74" s="45"/>
-      <c r="G74" s="45"/>
-      <c r="H74" s="45"/>
-      <c r="I74" s="45"/>
-    </row>
-    <row r="75" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="45"/>
-      <c r="B75" s="46"/>
-      <c r="C75" s="45"/>
-      <c r="D75" s="46"/>
-      <c r="E75" s="45"/>
-      <c r="F75" s="51"/>
-      <c r="G75" s="45"/>
-      <c r="H75" s="45"/>
-      <c r="I75" s="48"/>
-    </row>
-    <row r="76" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="45"/>
-      <c r="B76" s="46"/>
-      <c r="C76" s="45"/>
-      <c r="D76" s="46"/>
-      <c r="E76" s="45"/>
-      <c r="F76" s="51"/>
-      <c r="G76" s="45"/>
-      <c r="H76" s="45"/>
-      <c r="I76" s="48"/>
-    </row>
-    <row r="77" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="45"/>
-      <c r="B77" s="46"/>
-      <c r="C77" s="45"/>
-      <c r="D77" s="46"/>
-      <c r="E77" s="45"/>
-      <c r="F77" s="51"/>
-      <c r="G77" s="45"/>
-      <c r="H77" s="45"/>
-      <c r="I77" s="45"/>
-    </row>
-    <row r="78" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="45"/>
-      <c r="B78" s="46"/>
-      <c r="C78" s="45"/>
-      <c r="D78" s="46"/>
-      <c r="E78" s="45"/>
-      <c r="F78" s="45"/>
-      <c r="G78" s="45"/>
-      <c r="H78" s="45"/>
-      <c r="I78" s="45"/>
-    </row>
-    <row r="79" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="45"/>
-      <c r="B79" s="46"/>
-      <c r="C79" s="45"/>
-      <c r="D79" s="46"/>
-      <c r="E79" s="45"/>
-      <c r="F79" s="45"/>
-      <c r="G79" s="45"/>
-      <c r="H79" s="45"/>
-      <c r="I79" s="45"/>
-    </row>
-    <row r="80" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="45"/>
-      <c r="B80" s="46"/>
-      <c r="C80" s="45"/>
-      <c r="D80" s="46"/>
-      <c r="E80" s="45"/>
-      <c r="F80" s="45"/>
-      <c r="G80" s="45"/>
-      <c r="H80" s="45"/>
-      <c r="I80" s="45"/>
-    </row>
-    <row r="81" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="45"/>
-      <c r="B81" s="46"/>
-      <c r="C81" s="45"/>
-      <c r="D81" s="46"/>
-      <c r="E81" s="45"/>
-      <c r="F81" s="45"/>
-      <c r="G81" s="45"/>
-      <c r="H81" s="45"/>
-      <c r="I81" s="45"/>
-    </row>
-    <row r="82" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="45"/>
-      <c r="B82" s="46"/>
-      <c r="C82" s="45"/>
-      <c r="D82" s="46"/>
-      <c r="E82" s="45"/>
-      <c r="F82" s="45"/>
-      <c r="G82" s="45"/>
-      <c r="H82" s="45"/>
-      <c r="I82" s="45"/>
-    </row>
-    <row r="83" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="45"/>
-      <c r="B83" s="46"/>
-      <c r="C83" s="45"/>
-      <c r="D83" s="46"/>
-      <c r="E83" s="45"/>
-      <c r="F83" s="45"/>
-      <c r="G83" s="45"/>
-      <c r="H83" s="45"/>
-      <c r="I83" s="45"/>
-    </row>
-    <row r="84" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="45"/>
-      <c r="B84" s="46"/>
-      <c r="C84" s="45"/>
-      <c r="D84" s="46"/>
-      <c r="E84" s="45"/>
-      <c r="F84" s="51"/>
-      <c r="G84" s="45"/>
-      <c r="H84" s="45"/>
-      <c r="I84" s="45"/>
-    </row>
-    <row r="85" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="45"/>
-      <c r="B85" s="46"/>
-      <c r="C85" s="45"/>
-      <c r="D85" s="46"/>
-      <c r="E85" s="45"/>
-      <c r="F85" s="51"/>
-      <c r="G85" s="45"/>
-      <c r="H85" s="45"/>
-      <c r="I85" s="45"/>
-    </row>
-    <row r="86" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="45"/>
-      <c r="B86" s="46"/>
-      <c r="C86" s="45"/>
-      <c r="D86" s="46"/>
-      <c r="E86" s="45"/>
-      <c r="F86" s="45"/>
-      <c r="G86" s="45"/>
-      <c r="H86" s="45"/>
-      <c r="I86" s="45"/>
-    </row>
-    <row r="87" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="45"/>
-      <c r="B87" s="46"/>
-      <c r="C87" s="45"/>
-      <c r="D87" s="46"/>
-      <c r="E87" s="45"/>
-      <c r="F87" s="51"/>
-      <c r="G87" s="45"/>
-      <c r="H87" s="45"/>
-      <c r="I87" s="45"/>
-    </row>
-    <row r="88" spans="1:9" s="4" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="45"/>
-      <c r="B88" s="46"/>
-      <c r="C88" s="45"/>
-      <c r="D88" s="46"/>
-      <c r="E88" s="45"/>
-      <c r="F88" s="51"/>
-      <c r="G88" s="45"/>
-      <c r="H88" s="45"/>
-      <c r="I88" s="45"/>
-    </row>
-    <row r="89" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" s="18" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="14"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="14"/>
+    </row>
+    <row r="18" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="14"/>
+    </row>
+    <row r="19" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="14"/>
+      <c r="B19" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="16"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="14"/>
+      <c r="B20" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H20" s="17"/>
+      <c r="I20" s="14"/>
+    </row>
+    <row r="21" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="14"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="14"/>
+    </row>
+    <row r="22" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="14"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="14"/>
+    </row>
+    <row r="23" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="14"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="14"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="14"/>
+    </row>
+    <row r="25" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="14"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="14"/>
+    </row>
+    <row r="26" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="14"/>
+      <c r="B26" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H26" s="17"/>
+      <c r="I26" s="14"/>
+    </row>
+    <row r="27" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="I27" s="14"/>
+    </row>
+    <row r="28" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+    </row>
+    <row r="29" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+    </row>
+    <row r="30" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+    </row>
+    <row r="31" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+    </row>
+    <row r="32" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+    </row>
+    <row r="33" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+    </row>
+    <row r="34" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+    </row>
+    <row r="35" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+    </row>
+    <row r="36" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+    </row>
+    <row r="37" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+    </row>
+    <row r="38" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+    </row>
+    <row r="39" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+    </row>
+    <row r="40" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+    </row>
+    <row r="41" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+    </row>
+    <row r="43" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+    </row>
+    <row r="45" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+    </row>
+    <row r="50" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+    </row>
+    <row r="51" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+    </row>
+    <row r="52" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+    </row>
+    <row r="53" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+    </row>
+    <row r="54" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+    </row>
+    <row r="55" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+    </row>
+    <row r="56" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+    </row>
+    <row r="57" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+    </row>
+    <row r="58" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+    </row>
+    <row r="59" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+    </row>
+    <row r="60" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+    </row>
+    <row r="61" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+    </row>
+    <row r="62" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+    </row>
+    <row r="63" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+    </row>
+    <row r="64" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
+    </row>
+    <row r="65" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+      <c r="H65" s="3"/>
+    </row>
+    <row r="66" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
+    </row>
+    <row r="67" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="H67" s="3"/>
+    </row>
+    <row r="68" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
+    </row>
+    <row r="69" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+    </row>
+    <row r="70" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+    </row>
+    <row r="71" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="H71" s="3"/>
+    </row>
+    <row r="72" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="3"/>
+    </row>
+    <row r="73" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3"/>
+    </row>
+    <row r="74" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
+    </row>
+    <row r="75" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+    </row>
+    <row r="76" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
+    </row>
+    <row r="77" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3"/>
+    </row>
+    <row r="78" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3"/>
+    </row>
+    <row r="79" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+    </row>
+    <row r="80" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E80" s="3"/>
+      <c r="F80" s="3"/>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+    </row>
+    <row r="81" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+    </row>
+    <row r="82" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
+      <c r="G82" s="3"/>
+      <c r="H82" s="3"/>
+    </row>
+    <row r="83" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
+      <c r="H83" s="3"/>
+    </row>
+    <row r="84" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
+    </row>
+    <row r="85" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
+    </row>
+    <row r="86" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3"/>
+    </row>
+    <row r="87" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+    </row>
+    <row r="88" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+      <c r="G88" s="3"/>
+      <c r="H88" s="3"/>
+    </row>
+    <row r="89" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
     </row>
-    <row r="90" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="90" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E90" s="3"/>
       <c r="F90" s="3"/>
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
     </row>
-    <row r="91" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
     </row>
-    <row r="92" spans="1:9" s="18" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A92" s="14"/>
-      <c r="B92" s="15"/>
-      <c r="C92" s="16"/>
-      <c r="D92" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E92" s="17"/>
-      <c r="F92" s="17"/>
-      <c r="G92" s="17"/>
-      <c r="H92" s="17"/>
-      <c r="I92" s="14"/>
-    </row>
-    <row r="93" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A93" s="14"/>
-      <c r="B93" s="15"/>
-      <c r="C93" s="16"/>
-      <c r="D93" s="15"/>
-      <c r="E93" s="17"/>
-      <c r="F93" s="17"/>
-      <c r="G93" s="17"/>
-      <c r="H93" s="17"/>
-      <c r="I93" s="14"/>
-    </row>
-    <row r="94" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A94" s="14"/>
-      <c r="B94" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C94" s="16"/>
-      <c r="D94" s="15"/>
-      <c r="E94" s="17"/>
-      <c r="F94" s="17"/>
-      <c r="G94" s="17"/>
-      <c r="H94" s="17"/>
-      <c r="I94" s="14"/>
-    </row>
-    <row r="95" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A95" s="14"/>
-      <c r="B95" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C95" s="16"/>
-      <c r="D95" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="E95" s="17"/>
-      <c r="F95" s="17"/>
-      <c r="G95" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="H95" s="17"/>
-      <c r="I95" s="14"/>
-    </row>
-    <row r="96" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A96" s="14"/>
-      <c r="B96" s="15"/>
-      <c r="C96" s="16"/>
-      <c r="D96" s="15"/>
-      <c r="E96" s="17"/>
-      <c r="F96" s="17"/>
-      <c r="G96" s="17"/>
-      <c r="H96" s="17"/>
-      <c r="I96" s="14"/>
-    </row>
-    <row r="97" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A97" s="14"/>
-      <c r="B97" s="15"/>
-      <c r="C97" s="16"/>
-      <c r="D97" s="15"/>
-      <c r="E97" s="17"/>
-      <c r="F97" s="17"/>
-      <c r="G97" s="17"/>
-      <c r="H97" s="17"/>
-      <c r="I97" s="14"/>
-    </row>
-    <row r="98" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A98" s="14"/>
-      <c r="B98" s="15"/>
-      <c r="C98" s="16"/>
-      <c r="D98" s="15"/>
-      <c r="E98" s="17"/>
-      <c r="F98" s="17"/>
-      <c r="G98" s="17"/>
-      <c r="H98" s="17"/>
-      <c r="I98" s="14"/>
-    </row>
-    <row r="99" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A99" s="14"/>
-      <c r="B99" s="15"/>
-      <c r="C99" s="16"/>
-      <c r="D99" s="15"/>
-      <c r="E99" s="17"/>
-      <c r="F99" s="17"/>
-      <c r="G99" s="17"/>
-      <c r="H99" s="17"/>
-      <c r="I99" s="14"/>
-    </row>
-    <row r="100" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A100" s="14"/>
-      <c r="B100" s="15"/>
-      <c r="C100" s="16"/>
-      <c r="D100" s="15"/>
-      <c r="E100" s="17"/>
-      <c r="F100" s="17"/>
-      <c r="G100" s="17"/>
-      <c r="H100" s="17"/>
-      <c r="I100" s="14"/>
-    </row>
-    <row r="101" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A101" s="14"/>
-      <c r="B101" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C101" s="16"/>
-      <c r="D101" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E101" s="17"/>
-      <c r="F101" s="17"/>
-      <c r="G101" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="H101" s="17"/>
-      <c r="I101" s="14"/>
-    </row>
-    <row r="102" spans="1:9" s="18" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A102" s="14"/>
-      <c r="C102" s="14"/>
-      <c r="I102" s="14"/>
-    </row>
-    <row r="103" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
+    </row>
+    <row r="93" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
+    </row>
+    <row r="94" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
+    </row>
+    <row r="95" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
+    </row>
+    <row r="96" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3"/>
+    </row>
+    <row r="97" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+    </row>
+    <row r="98" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+    </row>
+    <row r="99" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3"/>
+      <c r="H99" s="3"/>
+    </row>
+    <row r="100" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="3"/>
+      <c r="H100" s="3"/>
+    </row>
+    <row r="101" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E101" s="3"/>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+    </row>
+    <row r="102" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E102" s="3"/>
+      <c r="F102" s="3"/>
+      <c r="G102" s="3"/>
+      <c r="H102" s="3"/>
+    </row>
+    <row r="103" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E103" s="3"/>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
       <c r="H103" s="3"/>
     </row>
-    <row r="104" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="104" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
       <c r="G104" s="3"/>
       <c r="H104" s="3"/>
     </row>
-    <row r="105" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="105" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E105" s="3"/>
       <c r="F105" s="3"/>
       <c r="G105" s="3"/>
       <c r="H105" s="3"/>
     </row>
-    <row r="106" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="106" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E106" s="3"/>
       <c r="F106" s="3"/>
       <c r="G106" s="3"/>
       <c r="H106" s="3"/>
     </row>
-    <row r="107" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="107" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E107" s="3"/>
       <c r="F107" s="3"/>
       <c r="G107" s="3"/>
       <c r="H107" s="3"/>
     </row>
-    <row r="108" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="108" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E108" s="3"/>
       <c r="F108" s="3"/>
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
     </row>
-    <row r="109" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="109" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E109" s="3"/>
       <c r="F109" s="3"/>
       <c r="G109" s="3"/>
       <c r="H109" s="3"/>
     </row>
-    <row r="110" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="110" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E110" s="3"/>
       <c r="F110" s="3"/>
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
     </row>
-    <row r="111" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="111" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E111" s="3"/>
       <c r="F111" s="3"/>
       <c r="G111" s="3"/>
       <c r="H111" s="3"/>
     </row>
-    <row r="112" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="112" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E112" s="3"/>
       <c r="F112" s="3"/>
       <c r="G112" s="3"/>
@@ -7149,456 +6790,6 @@
       <c r="F925" s="3"/>
       <c r="G925" s="3"/>
       <c r="H925" s="3"/>
-    </row>
-    <row r="926" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E926" s="3"/>
-      <c r="F926" s="3"/>
-      <c r="G926" s="3"/>
-      <c r="H926" s="3"/>
-    </row>
-    <row r="927" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E927" s="3"/>
-      <c r="F927" s="3"/>
-      <c r="G927" s="3"/>
-      <c r="H927" s="3"/>
-    </row>
-    <row r="928" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E928" s="3"/>
-      <c r="F928" s="3"/>
-      <c r="G928" s="3"/>
-      <c r="H928" s="3"/>
-    </row>
-    <row r="929" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E929" s="3"/>
-      <c r="F929" s="3"/>
-      <c r="G929" s="3"/>
-      <c r="H929" s="3"/>
-    </row>
-    <row r="930" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E930" s="3"/>
-      <c r="F930" s="3"/>
-      <c r="G930" s="3"/>
-      <c r="H930" s="3"/>
-    </row>
-    <row r="931" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E931" s="3"/>
-      <c r="F931" s="3"/>
-      <c r="G931" s="3"/>
-      <c r="H931" s="3"/>
-    </row>
-    <row r="932" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E932" s="3"/>
-      <c r="F932" s="3"/>
-      <c r="G932" s="3"/>
-      <c r="H932" s="3"/>
-    </row>
-    <row r="933" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E933" s="3"/>
-      <c r="F933" s="3"/>
-      <c r="G933" s="3"/>
-      <c r="H933" s="3"/>
-    </row>
-    <row r="934" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E934" s="3"/>
-      <c r="F934" s="3"/>
-      <c r="G934" s="3"/>
-      <c r="H934" s="3"/>
-    </row>
-    <row r="935" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E935" s="3"/>
-      <c r="F935" s="3"/>
-      <c r="G935" s="3"/>
-      <c r="H935" s="3"/>
-    </row>
-    <row r="936" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E936" s="3"/>
-      <c r="F936" s="3"/>
-      <c r="G936" s="3"/>
-      <c r="H936" s="3"/>
-    </row>
-    <row r="937" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E937" s="3"/>
-      <c r="F937" s="3"/>
-      <c r="G937" s="3"/>
-      <c r="H937" s="3"/>
-    </row>
-    <row r="938" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E938" s="3"/>
-      <c r="F938" s="3"/>
-      <c r="G938" s="3"/>
-      <c r="H938" s="3"/>
-    </row>
-    <row r="939" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E939" s="3"/>
-      <c r="F939" s="3"/>
-      <c r="G939" s="3"/>
-      <c r="H939" s="3"/>
-    </row>
-    <row r="940" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E940" s="3"/>
-      <c r="F940" s="3"/>
-      <c r="G940" s="3"/>
-      <c r="H940" s="3"/>
-    </row>
-    <row r="941" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E941" s="3"/>
-      <c r="F941" s="3"/>
-      <c r="G941" s="3"/>
-      <c r="H941" s="3"/>
-    </row>
-    <row r="942" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E942" s="3"/>
-      <c r="F942" s="3"/>
-      <c r="G942" s="3"/>
-      <c r="H942" s="3"/>
-    </row>
-    <row r="943" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E943" s="3"/>
-      <c r="F943" s="3"/>
-      <c r="G943" s="3"/>
-      <c r="H943" s="3"/>
-    </row>
-    <row r="944" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E944" s="3"/>
-      <c r="F944" s="3"/>
-      <c r="G944" s="3"/>
-      <c r="H944" s="3"/>
-    </row>
-    <row r="945" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E945" s="3"/>
-      <c r="F945" s="3"/>
-      <c r="G945" s="3"/>
-      <c r="H945" s="3"/>
-    </row>
-    <row r="946" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E946" s="3"/>
-      <c r="F946" s="3"/>
-      <c r="G946" s="3"/>
-      <c r="H946" s="3"/>
-    </row>
-    <row r="947" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E947" s="3"/>
-      <c r="F947" s="3"/>
-      <c r="G947" s="3"/>
-      <c r="H947" s="3"/>
-    </row>
-    <row r="948" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E948" s="3"/>
-      <c r="F948" s="3"/>
-      <c r="G948" s="3"/>
-      <c r="H948" s="3"/>
-    </row>
-    <row r="949" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E949" s="3"/>
-      <c r="F949" s="3"/>
-      <c r="G949" s="3"/>
-      <c r="H949" s="3"/>
-    </row>
-    <row r="950" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E950" s="3"/>
-      <c r="F950" s="3"/>
-      <c r="G950" s="3"/>
-      <c r="H950" s="3"/>
-    </row>
-    <row r="951" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E951" s="3"/>
-      <c r="F951" s="3"/>
-      <c r="G951" s="3"/>
-      <c r="H951" s="3"/>
-    </row>
-    <row r="952" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E952" s="3"/>
-      <c r="F952" s="3"/>
-      <c r="G952" s="3"/>
-      <c r="H952" s="3"/>
-    </row>
-    <row r="953" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E953" s="3"/>
-      <c r="F953" s="3"/>
-      <c r="G953" s="3"/>
-      <c r="H953" s="3"/>
-    </row>
-    <row r="954" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E954" s="3"/>
-      <c r="F954" s="3"/>
-      <c r="G954" s="3"/>
-      <c r="H954" s="3"/>
-    </row>
-    <row r="955" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E955" s="3"/>
-      <c r="F955" s="3"/>
-      <c r="G955" s="3"/>
-      <c r="H955" s="3"/>
-    </row>
-    <row r="956" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E956" s="3"/>
-      <c r="F956" s="3"/>
-      <c r="G956" s="3"/>
-      <c r="H956" s="3"/>
-    </row>
-    <row r="957" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E957" s="3"/>
-      <c r="F957" s="3"/>
-      <c r="G957" s="3"/>
-      <c r="H957" s="3"/>
-    </row>
-    <row r="958" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E958" s="3"/>
-      <c r="F958" s="3"/>
-      <c r="G958" s="3"/>
-      <c r="H958" s="3"/>
-    </row>
-    <row r="959" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E959" s="3"/>
-      <c r="F959" s="3"/>
-      <c r="G959" s="3"/>
-      <c r="H959" s="3"/>
-    </row>
-    <row r="960" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E960" s="3"/>
-      <c r="F960" s="3"/>
-      <c r="G960" s="3"/>
-      <c r="H960" s="3"/>
-    </row>
-    <row r="961" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E961" s="3"/>
-      <c r="F961" s="3"/>
-      <c r="G961" s="3"/>
-      <c r="H961" s="3"/>
-    </row>
-    <row r="962" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E962" s="3"/>
-      <c r="F962" s="3"/>
-      <c r="G962" s="3"/>
-      <c r="H962" s="3"/>
-    </row>
-    <row r="963" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E963" s="3"/>
-      <c r="F963" s="3"/>
-      <c r="G963" s="3"/>
-      <c r="H963" s="3"/>
-    </row>
-    <row r="964" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E964" s="3"/>
-      <c r="F964" s="3"/>
-      <c r="G964" s="3"/>
-      <c r="H964" s="3"/>
-    </row>
-    <row r="965" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E965" s="3"/>
-      <c r="F965" s="3"/>
-      <c r="G965" s="3"/>
-      <c r="H965" s="3"/>
-    </row>
-    <row r="966" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E966" s="3"/>
-      <c r="F966" s="3"/>
-      <c r="G966" s="3"/>
-      <c r="H966" s="3"/>
-    </row>
-    <row r="967" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E967" s="3"/>
-      <c r="F967" s="3"/>
-      <c r="G967" s="3"/>
-      <c r="H967" s="3"/>
-    </row>
-    <row r="968" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E968" s="3"/>
-      <c r="F968" s="3"/>
-      <c r="G968" s="3"/>
-      <c r="H968" s="3"/>
-    </row>
-    <row r="969" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E969" s="3"/>
-      <c r="F969" s="3"/>
-      <c r="G969" s="3"/>
-      <c r="H969" s="3"/>
-    </row>
-    <row r="970" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E970" s="3"/>
-      <c r="F970" s="3"/>
-      <c r="G970" s="3"/>
-      <c r="H970" s="3"/>
-    </row>
-    <row r="971" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E971" s="3"/>
-      <c r="F971" s="3"/>
-      <c r="G971" s="3"/>
-      <c r="H971" s="3"/>
-    </row>
-    <row r="972" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E972" s="3"/>
-      <c r="F972" s="3"/>
-      <c r="G972" s="3"/>
-      <c r="H972" s="3"/>
-    </row>
-    <row r="973" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E973" s="3"/>
-      <c r="F973" s="3"/>
-      <c r="G973" s="3"/>
-      <c r="H973" s="3"/>
-    </row>
-    <row r="974" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E974" s="3"/>
-      <c r="F974" s="3"/>
-      <c r="G974" s="3"/>
-      <c r="H974" s="3"/>
-    </row>
-    <row r="975" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E975" s="3"/>
-      <c r="F975" s="3"/>
-      <c r="G975" s="3"/>
-      <c r="H975" s="3"/>
-    </row>
-    <row r="976" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E976" s="3"/>
-      <c r="F976" s="3"/>
-      <c r="G976" s="3"/>
-      <c r="H976" s="3"/>
-    </row>
-    <row r="977" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E977" s="3"/>
-      <c r="F977" s="3"/>
-      <c r="G977" s="3"/>
-      <c r="H977" s="3"/>
-    </row>
-    <row r="978" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E978" s="3"/>
-      <c r="F978" s="3"/>
-      <c r="G978" s="3"/>
-      <c r="H978" s="3"/>
-    </row>
-    <row r="979" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E979" s="3"/>
-      <c r="F979" s="3"/>
-      <c r="G979" s="3"/>
-      <c r="H979" s="3"/>
-    </row>
-    <row r="980" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E980" s="3"/>
-      <c r="F980" s="3"/>
-      <c r="G980" s="3"/>
-      <c r="H980" s="3"/>
-    </row>
-    <row r="981" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E981" s="3"/>
-      <c r="F981" s="3"/>
-      <c r="G981" s="3"/>
-      <c r="H981" s="3"/>
-    </row>
-    <row r="982" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E982" s="3"/>
-      <c r="F982" s="3"/>
-      <c r="G982" s="3"/>
-      <c r="H982" s="3"/>
-    </row>
-    <row r="983" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E983" s="3"/>
-      <c r="F983" s="3"/>
-      <c r="G983" s="3"/>
-      <c r="H983" s="3"/>
-    </row>
-    <row r="984" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E984" s="3"/>
-      <c r="F984" s="3"/>
-      <c r="G984" s="3"/>
-      <c r="H984" s="3"/>
-    </row>
-    <row r="985" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E985" s="3"/>
-      <c r="F985" s="3"/>
-      <c r="G985" s="3"/>
-      <c r="H985" s="3"/>
-    </row>
-    <row r="986" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E986" s="3"/>
-      <c r="F986" s="3"/>
-      <c r="G986" s="3"/>
-      <c r="H986" s="3"/>
-    </row>
-    <row r="987" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E987" s="3"/>
-      <c r="F987" s="3"/>
-      <c r="G987" s="3"/>
-      <c r="H987" s="3"/>
-    </row>
-    <row r="988" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E988" s="3"/>
-      <c r="F988" s="3"/>
-      <c r="G988" s="3"/>
-      <c r="H988" s="3"/>
-    </row>
-    <row r="989" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E989" s="3"/>
-      <c r="F989" s="3"/>
-      <c r="G989" s="3"/>
-      <c r="H989" s="3"/>
-    </row>
-    <row r="990" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E990" s="3"/>
-      <c r="F990" s="3"/>
-      <c r="G990" s="3"/>
-      <c r="H990" s="3"/>
-    </row>
-    <row r="991" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E991" s="3"/>
-      <c r="F991" s="3"/>
-      <c r="G991" s="3"/>
-      <c r="H991" s="3"/>
-    </row>
-    <row r="992" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E992" s="3"/>
-      <c r="F992" s="3"/>
-      <c r="G992" s="3"/>
-      <c r="H992" s="3"/>
-    </row>
-    <row r="993" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E993" s="3"/>
-      <c r="F993" s="3"/>
-      <c r="G993" s="3"/>
-      <c r="H993" s="3"/>
-    </row>
-    <row r="994" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E994" s="3"/>
-      <c r="F994" s="3"/>
-      <c r="G994" s="3"/>
-      <c r="H994" s="3"/>
-    </row>
-    <row r="995" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E995" s="3"/>
-      <c r="F995" s="3"/>
-      <c r="G995" s="3"/>
-      <c r="H995" s="3"/>
-    </row>
-    <row r="996" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E996" s="3"/>
-      <c r="F996" s="3"/>
-      <c r="G996" s="3"/>
-      <c r="H996" s="3"/>
-    </row>
-    <row r="997" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E997" s="3"/>
-      <c r="F997" s="3"/>
-      <c r="G997" s="3"/>
-      <c r="H997" s="3"/>
-    </row>
-    <row r="998" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E998" s="3"/>
-      <c r="F998" s="3"/>
-      <c r="G998" s="3"/>
-      <c r="H998" s="3"/>
-    </row>
-    <row r="999" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E999" s="3"/>
-      <c r="F999" s="3"/>
-      <c r="G999" s="3"/>
-      <c r="H999" s="3"/>
-    </row>
-    <row r="1000" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E1000" s="3"/>
-      <c r="F1000" s="3"/>
-      <c r="G1000" s="3"/>
-      <c r="H1000" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="17">

</xml_diff>

<commit_message>
feat: add initial spreadsheet templates for faculty and study program reporting
</commit_message>
<xml_diff>
--- a/resources/templates/Laporan Pelaksanaan Perkuliahan Prodi Ilmu Komputer.xlsx
+++ b/resources/templates/Laporan Pelaksanaan Perkuliahan Prodi Ilmu Komputer.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -118,7 +118,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -184,12 +184,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -465,7 +459,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -495,57 +489,31 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -589,28 +557,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1048,7 +1018,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:I925"/>
   <sheetFormatPr defaultColWidth="59.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="59.6328125" style="6"/>
@@ -1072,104 +1042,104 @@
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9" s="4" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="37" t="s">
+      <c r="A2" s="21"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="38"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="28"/>
     </row>
     <row r="3" spans="1:9" s="4" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="33"/>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="39"/>
+      <c r="A3" s="23"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" spans="1:9" s="4" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="33"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="39"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="29"/>
     </row>
     <row r="5" spans="1:9" s="4" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="40" t="s">
+      <c r="A5" s="23"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="39"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="29"/>
     </row>
     <row r="6" spans="1:9" s="4" customFormat="1" ht="17.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="33"/>
-      <c r="B6" s="34"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="41" t="s">
+      <c r="A6" s="23"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="39"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="29"/>
     </row>
     <row r="7" spans="1:9" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="42" t="s">
+      <c r="A7" s="23"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="39"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="29"/>
     </row>
     <row r="8" spans="1:9" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="33"/>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="42" t="s">
+      <c r="A8" s="23"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="39"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="29"/>
     </row>
     <row r="9" spans="1:9" s="4" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="35"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="43" t="s">
+      <c r="A9" s="25"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="44"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="34"/>
     </row>
     <row r="10" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="7"/>
@@ -1183,30 +1153,30 @@
       <c r="I10" s="10"/>
     </row>
     <row r="11" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="27"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="41"/>
     </row>
     <row r="12" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="27"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="41"/>
     </row>
     <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="7"/>
@@ -1220,46 +1190,46 @@
       <c r="I13" s="10"/>
     </row>
     <row r="14" spans="1:9" s="11" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="24"/>
-      <c r="I14" s="28" t="s">
+      <c r="H14" s="38"/>
+      <c r="I14" s="42" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="11" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="A15" s="43"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
       <c r="G15" s="12" t="s">
         <v>16</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="30"/>
+      <c r="I15" s="44"/>
     </row>
     <row r="16" spans="1:9" s="4" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
@@ -1433,31 +1403,31 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
     </row>
-    <row r="33" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
     </row>
-    <row r="34" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
     </row>
-    <row r="35" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
     </row>
-    <row r="36" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
     </row>
-    <row r="37" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="5:8" ht="12.5" x14ac:dyDescent="0.25">
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -6793,13 +6763,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A2:C9"/>
-    <mergeCell ref="D2:I4"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="D6:I6"/>
-    <mergeCell ref="D7:I7"/>
-    <mergeCell ref="D8:I8"/>
-    <mergeCell ref="D9:I9"/>
     <mergeCell ref="F14:F15"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="A11:I11"/>
@@ -6810,6 +6773,13 @@
     <mergeCell ref="D14:D15"/>
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="I14:I15"/>
+    <mergeCell ref="A2:C9"/>
+    <mergeCell ref="D2:I4"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="D8:I8"/>
+    <mergeCell ref="D9:I9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D9" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>